<commit_message>
gestione fornitori con più cc
</commit_message>
<xml_diff>
--- a/SmartCheckIBAN/ExportSCI.xlsx
+++ b/SmartCheckIBAN/ExportSCI.xlsx
@@ -11,12 +11,15 @@
     <sheet name="Foglio2" sheetId="2" r:id="rId2"/>
     <sheet name="Foglio3" sheetId="3" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Foglio1!$A$1:$L$1</definedName>
+  </definedNames>
   <calcPr calcId="125725"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="10">
   <si>
     <t>Codice Fornitore</t>
   </si>
@@ -36,13 +39,16 @@
     <t>IBAN</t>
   </si>
   <si>
-    <t>Data Controllo</t>
-  </si>
-  <si>
     <t>Esito</t>
   </si>
   <si>
     <t>Note</t>
+  </si>
+  <si>
+    <t>Data Ultimo Controllo</t>
+  </si>
+  <si>
+    <t>Data Penultimo Controllo</t>
   </si>
 </sst>
 </file>
@@ -385,7 +391,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.85546875" bestFit="1" customWidth="1"/>
@@ -394,9 +400,10 @@
     <col min="4" max="4" width="14.85546875" customWidth="1"/>
     <col min="5" max="5" width="30.140625" customWidth="1"/>
     <col min="7" max="7" width="13.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.85546875" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="2" customFormat="1" ht="18.75">
+    <row r="1" spans="1:12" s="2" customFormat="1" ht="18.75">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -416,16 +423,26 @@
         <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
-        <v>8</v>
+      <c r="J1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:L1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>